<commit_message>
still trying to fix
</commit_message>
<xml_diff>
--- a/master_template.xlsx
+++ b/master_template.xlsx
@@ -8,17 +8,16 @@
   </bookViews>
   <sheets>
     <sheet name="digestion_page" sheetId="1" r:id="rId1"/>
-    <sheet name="200126511" sheetId="2" r:id="rId2"/>
-    <sheet name="200126512" sheetId="3" r:id="rId3"/>
-    <sheet name="200126513" sheetId="4" r:id="rId4"/>
-    <sheet name="formula_page" sheetId="5" r:id="rId5"/>
+    <sheet name="2001265" sheetId="2" r:id="rId2"/>
+    <sheet name="2001266" sheetId="3" r:id="rId3"/>
+    <sheet name="formula_page" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="44">
   <si>
     <t>Date:</t>
   </si>
@@ -53,22 +52,16 @@
     <t>volume (mL)</t>
   </si>
   <si>
-    <t>200126511_1</t>
-  </si>
-  <si>
-    <t>200126511_2</t>
-  </si>
-  <si>
-    <t>200126512_1</t>
-  </si>
-  <si>
-    <t>200126512_2</t>
-  </si>
-  <si>
-    <t>200126513_1</t>
-  </si>
-  <si>
-    <t>200126513_2</t>
+    <t>2001265_1</t>
+  </si>
+  <si>
+    <t>2001265_2</t>
+  </si>
+  <si>
+    <t>2001266_1</t>
+  </si>
+  <si>
+    <t>2001266_2</t>
   </si>
   <si>
     <t>Cr6</t>
@@ -107,7 +100,7 @@
     <t>Cr3 titration analysis</t>
   </si>
   <si>
-    <t>200126511</t>
+    <t>2001265</t>
   </si>
   <si>
     <t>cr3 result:</t>
@@ -116,10 +109,7 @@
     <t>Note(s):</t>
   </si>
   <si>
-    <t>200126512</t>
-  </si>
-  <si>
-    <t>200126513</t>
+    <t>2001266</t>
   </si>
   <si>
     <t>A = crucible</t>
@@ -578,10 +568,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -591,7 +581,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -671,185 +661,143 @@
       <c r="B13" s="6"/>
       <c r="C13" s="5"/>
     </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="4" t="s">
+    <row r="16" spans="1:3">
+      <c r="A16" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="5"/>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="5"/>
+      <c r="C17" s="5"/>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
+      <c r="A18" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>17</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="B19" s="5"/>
       <c r="C19" s="5"/>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
+        <v>8</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B21" s="5"/>
+        <v>11</v>
+      </c>
+      <c r="B21" s="6"/>
       <c r="C21" s="5"/>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>10</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="5"/>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="5"/>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="5"/>
     </row>
-    <row r="25" spans="1:3">
-      <c r="A25" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="5"/>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="5"/>
-    </row>
     <row r="27" spans="1:3">
-      <c r="A27" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="5"/>
+      <c r="A27" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B28" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="6"/>
       <c r="C28" s="5"/>
     </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
+    </row>
     <row r="31" spans="1:3">
-      <c r="A31" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
+      <c r="A31" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>18</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B32" s="6"/>
       <c r="C32" s="5"/>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B33" s="5"/>
+        <v>12</v>
+      </c>
+      <c r="B33" s="6"/>
       <c r="C33" s="5"/>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B34" s="5"/>
+        <v>13</v>
+      </c>
+      <c r="B34" s="6"/>
       <c r="C34" s="5"/>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B36" s="6"/>
-      <c r="C36" s="5"/>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B37" s="6"/>
-      <c r="C37" s="5"/>
-    </row>
-    <row r="38" spans="1:3">
-      <c r="A38" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B38" s="6"/>
-      <c r="C38" s="5"/>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B39" s="6"/>
-      <c r="C39" s="5"/>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B40" s="6"/>
-      <c r="C40" s="5"/>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B41" s="6"/>
-      <c r="C41" s="5"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -857,14 +805,14 @@
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
     <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -886,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -899,22 +847,22 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B5" s="7"/>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -928,7 +876,7 @@
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="G7" s="8">
-        <f>digestion_page!B36</f>
+        <f>digestion_page!B32</f>
         <v>0</v>
       </c>
     </row>
@@ -943,20 +891,20 @@
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
       <c r="G8" s="8">
-        <f>digestion_page!B37</f>
+        <f>digestion_page!B33</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="7"/>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="10">
@@ -966,7 +914,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="11">
@@ -976,22 +924,22 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B14" s="7"/>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -1005,7 +953,7 @@
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="G16" s="8">
-        <f>digestion_page!B23</f>
+        <f>digestion_page!B21</f>
         <v>0</v>
       </c>
     </row>
@@ -1020,20 +968,20 @@
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
       <c r="G17" s="8">
-        <f>digestion_page!B24</f>
+        <f>digestion_page!B22</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B19" s="9"/>
       <c r="C19" s="7"/>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="10">
@@ -1043,7 +991,7 @@
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="11">
@@ -1053,24 +1001,24 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B23" s="7"/>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="C24" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B25" s="5">
         <f>C12</f>
@@ -1083,7 +1031,7 @@
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B27" s="9"/>
       <c r="C27" s="10">
@@ -1093,7 +1041,7 @@
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B28" s="9"/>
       <c r="C28" s="11">
@@ -1103,7 +1051,7 @@
     </row>
     <row r="30" spans="1:7">
       <c r="B30" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C30" s="12"/>
       <c r="D30" s="12"/>
@@ -1167,7 +1115,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46146</v>
+        <v>46147</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -1180,22 +1128,22 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B5" s="7"/>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1209,7 +1157,7 @@
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="G7" s="8">
-        <f>digestion_page!B38</f>
+        <f>digestion_page!B34</f>
         <v>0</v>
       </c>
     </row>
@@ -1224,20 +1172,20 @@
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
       <c r="G8" s="8">
-        <f>digestion_page!B39</f>
+        <f>digestion_page!B35</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B10" s="9"/>
       <c r="C10" s="7"/>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="10">
@@ -1247,7 +1195,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="11">
@@ -1257,22 +1205,22 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B14" s="7"/>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>9</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -1286,7 +1234,7 @@
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="G16" s="8">
-        <f>digestion_page!B25</f>
+        <f>digestion_page!B23</f>
         <v>0</v>
       </c>
     </row>
@@ -1301,20 +1249,20 @@
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
       <c r="G17" s="8">
-        <f>digestion_page!B26</f>
+        <f>digestion_page!B24</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B19" s="9"/>
       <c r="C19" s="7"/>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="10">
@@ -1324,7 +1272,7 @@
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="11">
@@ -1334,24 +1282,24 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B23" s="7"/>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="C24" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B25" s="5">
         <f>C12</f>
@@ -1364,7 +1312,7 @@
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B27" s="9"/>
       <c r="C27" s="10">
@@ -1374,7 +1322,7 @@
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B28" s="9"/>
       <c r="C28" s="11">
@@ -1384,7 +1332,7 @@
     </row>
     <row r="30" spans="1:7">
       <c r="B30" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C30" s="12"/>
       <c r="D30" s="12"/>
@@ -1434,287 +1382,6 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G32"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2">
-        <v>46146</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="7"/>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="6">
-        <f>G7</f>
-        <v>0</v>
-      </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="G7" s="8">
-        <f>digestion_page!B40</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="6">
-        <f>G8</f>
-        <v>0</v>
-      </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="G8" s="8">
-        <f>digestion_page!B41</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="7"/>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="9"/>
-      <c r="C11" s="10">
-        <f>AVERAGE(D7:D8)*(10000)*(1/1)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="11">
-        <f>AVERAGE(D7:D8)*(1/1)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="7"/>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="6">
-        <f>G16</f>
-        <v>0</v>
-      </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="G16" s="8">
-        <f>digestion_page!B27</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="A17" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="6">
-        <f>G17</f>
-        <v>0</v>
-      </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="G17" s="8">
-        <f>digestion_page!B28</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="7"/>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="10">
-        <f>AVERAGE(D16:D17)*(10000)*(1/1)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="9"/>
-      <c r="C21" s="11">
-        <f>AVERAGE(D16:D17)*(1/1)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" s="7"/>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B25" s="5">
-        <f>C12</f>
-        <v>0</v>
-      </c>
-      <c r="C25" s="5">
-        <f>C21</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
-      <c r="A27" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B27" s="9"/>
-      <c r="C27" s="10">
-        <f>(C12-C21)*(10000)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="A28" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" s="9"/>
-      <c r="C28" s="11">
-        <f>(C12-C21)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="B30" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
-    </row>
-    <row r="31" spans="1:7">
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
-    </row>
-  </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C30:F32"/>
-  </mergeCells>
-  <conditionalFormatting sqref="C10">
-    <cfRule type="containsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(C10))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C19">
-    <cfRule type="containsBlanks" dxfId="0" priority="2">
-      <formula>LEN(TRIM(C19))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1723,67 +1390,67 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="13" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="13" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="13" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="13" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="13" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="13" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="13" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="13" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="13" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="13" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="13" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" s="13" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>